<commit_message>
Atualiza Taxas Antigas NTNB.xlsx (sync manual)
</commit_message>
<xml_diff>
--- a/Taxas Antigas NTNB.xlsx
+++ b/Taxas Antigas NTNB.xlsx
@@ -127,9 +127,9 @@
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="Yu Gothic Light"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="ç­çº¿ Light"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ§ÃÂ­ÃÂÃÂ§ÃÂºÃÂ¿ Light"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -162,9 +162,9 @@
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="Yu Gothic"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="ç­çº¿"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ§ÃÂ­ÃÂÃÂ§ÃÂºÃÂ¿"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -346,10 +346,10 @@
   <dimension ref="C2:D10"/>
   <cols>
     <col min="3" max="3" customWidth="1" width="12"/>
-    <col min="4" max="4" customWidth="1" width="11.42578125"/>
+    <col min="4" max="4" customWidth="1" width="11.375"/>
   </cols>
   <sheetData>
-    <row r="2">
+    <row r="2" ht="15.75" customHeight="1">
       <c r="C2" s="1">
         <v>46234</v>
       </c>
@@ -424,15 +424,15 @@
   <dimension ref="C2:AO10"/>
   <cols>
     <col min="3" max="3" customWidth="1" width="12"/>
-    <col min="4" max="4" customWidth="1" width="11.42578125"/>
-    <col min="24" max="24" customWidth="1" width="10.7109375"/>
-    <col min="28" max="28" customWidth="1" width="10.7109375"/>
-    <col min="32" max="32" customWidth="1" width="10.7109375"/>
-    <col min="36" max="36" customWidth="1" width="10.7109375"/>
-    <col min="40" max="40" customWidth="1" width="10.7109375"/>
+    <col min="4" max="4" customWidth="1" width="11.375"/>
+    <col min="24" max="24" customWidth="1" width="10.75"/>
+    <col min="28" max="28" customWidth="1" width="10.75"/>
+    <col min="32" max="32" customWidth="1" width="10.75"/>
+    <col min="36" max="36" customWidth="1" width="10.75"/>
+    <col min="40" max="40" customWidth="1" width="10.75"/>
   </cols>
   <sheetData>
-    <row r="2">
+    <row r="2" ht="15.75" customHeight="1">
       <c r="C2" s="1">
         <v>46021</v>
       </c>
@@ -909,20 +909,80 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="C2:T11"/>
+  <dimension ref="C2:CD11"/>
   <cols>
-    <col min="3" max="3" customWidth="1" width="11.28515625"/>
-    <col min="7" max="7" customWidth="1" width="11.28515625"/>
-    <col min="11" max="11" customWidth="1" width="11.28515625"/>
-    <col min="15" max="15" customWidth="1" width="11.28515625"/>
+    <col min="3" max="3" customWidth="1" width="11.25"/>
+    <col min="7" max="7" customWidth="1" width="11.25"/>
+    <col min="11" max="11" customWidth="1" width="11.25"/>
+    <col min="15" max="15" customWidth="1" width="11.25"/>
   </cols>
   <sheetData>
-    <row r="2">
-      <c r="S2">
-        <v>46265</v>
-      </c>
-    </row>
-    <row r="3">
+    <row r="2" ht="16.5" customHeight="1">
+      <c r="S2" s="3">
+        <v>46080</v>
+      </c>
+      <c r="W2" s="3">
+        <v>46097</v>
+      </c>
+      <c r="AA2" s="3">
+        <v>46112</v>
+      </c>
+      <c r="AE2" s="3">
+        <v>46120</v>
+      </c>
+      <c r="AH2" s="3">
+        <v>46129</v>
+      </c>
+      <c r="AL2" s="3">
+        <v>46142</v>
+      </c>
+      <c r="AP2" s="3">
+        <v>46157</v>
+      </c>
+      <c r="AS2" s="3">
+        <v>46171</v>
+      </c>
+      <c r="AV2" s="3">
+        <v>46188</v>
+      </c>
+      <c r="AY2" s="3">
+        <v>46203</v>
+      </c>
+      <c r="BB2" s="3">
+        <v>46217</v>
+      </c>
+      <c r="BE2" s="3">
+        <v>46234</v>
+      </c>
+      <c r="BH2" s="3">
+        <v>46252</v>
+      </c>
+      <c r="BN2" s="3">
+        <v>46280</v>
+      </c>
+      <c r="BQ2" s="3">
+        <v>46287</v>
+      </c>
+      <c r="BS2">
+        <v>46276</v>
+      </c>
+      <c r="BU2">
+        <v>46279</v>
+      </c>
+      <c r="BW2">
+        <v>46281</v>
+      </c>
+      <c r="BY2">
+        <v>46282</v>
+      </c>
+      <c r="CA2">
+        <v>46283</v>
+      </c>
+      <c r="CC2">
+        <v>46286</v>
+      </c>
+    </row>
+    <row r="3" ht="18.75" customHeight="1">
       <c r="C3" s="3">
         <v>46027</v>
       </c>
@@ -941,48 +1001,423 @@
       <c r="T3" t="str">
         <v>Taxa Atual</v>
       </c>
+      <c r="W3" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="X3" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="AA3" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="AB3" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="AE3" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="AF3" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="AH3" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="AI3" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="AL3" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="AM3" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="AP3" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="AQ3" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="AS3" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="AT3" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="AV3" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="AW3" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="AY3" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="AZ3" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="BB3" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="BC3" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="BE3" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="BF3" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="BH3" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="BI3" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="BK3" s="3">
+        <v>46265</v>
+      </c>
+      <c r="BN3" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="BO3" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="BQ3" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="BR3" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="BS3" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="BT3" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="BU3" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="BV3" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="BW3" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="BX3" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="BY3" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="BZ3" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="CA3" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="CB3" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="CC3" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="CD3" t="str">
+        <v>Taxa Atual</v>
+      </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="S4" t="str">
         <v>NTNB 2028</v>
       </c>
-      <c r="T4">
+      <c r="T4" s="2">
+        <v>0.0779</v>
+      </c>
+      <c r="W4" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="X4" s="2">
+        <v>0.0845</v>
+      </c>
+      <c r="AA4" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="AB4" s="2">
+        <v>0.078</v>
+      </c>
+      <c r="AE4" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="AF4" s="2">
+        <v>0.0779</v>
+      </c>
+      <c r="AH4" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="AI4" s="2">
+        <v>0.077</v>
+      </c>
+      <c r="AL4" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="AM4" s="2">
+        <v>0.0796</v>
+      </c>
+      <c r="AP4" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="AQ4" s="2">
+        <v>0.081</v>
+      </c>
+      <c r="AS4" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="AT4" s="2">
+        <v>0.0817</v>
+      </c>
+      <c r="AV4" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="AW4" s="2">
+        <v>0.0877</v>
+      </c>
+      <c r="AY4" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="AZ4" s="2">
+        <v>0.0889</v>
+      </c>
+      <c r="BB4" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="BC4" s="2">
+        <v>0.0855</v>
+      </c>
+      <c r="BE4" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="BF4" s="2">
+        <v>0.0847</v>
+      </c>
+      <c r="BH4" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="BI4" s="2">
+        <v>0.0822</v>
+      </c>
+      <c r="BK4" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="BL4" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="BN4" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="BO4" s="2">
+        <v>0.0753</v>
+      </c>
+      <c r="BQ4" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="BR4" s="2">
+        <v>0.0742</v>
+      </c>
+      <c r="BS4" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="BT4">
+        <v>0.075343</v>
+      </c>
+      <c r="BU4" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="BV4">
+        <v>0.07515100000000001</v>
+      </c>
+      <c r="BW4" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="BX4">
+        <v>0.074712</v>
+      </c>
+      <c r="BY4" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="BZ4">
+        <v>0.073636</v>
+      </c>
+      <c r="CA4" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="CB4">
+        <v>0.0733</v>
+      </c>
+      <c r="CC4" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="CD4">
+        <v>0.07377600000000001</v>
+      </c>
+    </row>
+    <row r="5" ht="18.75" customHeight="1">
+      <c r="C5" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="O5" t="str">
+        <v>Papel</v>
+      </c>
+      <c r="P5" t="str">
+        <v>Taxa Atual</v>
+      </c>
+      <c r="S5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="T5" s="2">
+        <v>0.0761</v>
+      </c>
+      <c r="W5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="X5" s="2">
+        <v>0.0825</v>
+      </c>
+      <c r="AA5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="AB5" s="2">
+        <v>0.0778</v>
+      </c>
+      <c r="AE5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="AF5" s="2">
+        <v>0.0775</v>
+      </c>
+      <c r="AH5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="AI5" s="2">
+        <v>0.0758</v>
+      </c>
+      <c r="AL5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="AM5" s="2">
+        <v>0.0785</v>
+      </c>
+      <c r="AP5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="AQ5" s="2">
+        <v>0.0804</v>
+      </c>
+      <c r="AS5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="AT5" s="2">
+        <v>0.0812</v>
+      </c>
+      <c r="AV5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="AW5" s="2">
+        <v>0.0859</v>
+      </c>
+      <c r="AY5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="AZ5" s="2">
+        <v>0.0864</v>
+      </c>
+      <c r="BB5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="BC5" s="2">
+        <v>0.0832</v>
+      </c>
+      <c r="BE5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="BF5" s="2">
+        <v>0.0823</v>
+      </c>
+      <c r="BH5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="BI5" s="2">
+        <v>0.0811</v>
+      </c>
+      <c r="BK5" t="str">
+        <v>NTNB 2028</v>
+      </c>
+      <c r="BL5" s="2">
         <v>0.0794</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="C5" t="str">
-        <v>Papel</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Taxa Atual</v>
-      </c>
-      <c r="G5" t="str">
-        <v>Papel</v>
-      </c>
-      <c r="H5" t="str">
-        <v>Taxa Atual</v>
-      </c>
-      <c r="K5" t="str">
-        <v>Papel</v>
-      </c>
-      <c r="L5" t="str">
-        <v>Taxa Atual</v>
-      </c>
-      <c r="O5" t="str">
-        <v>Papel</v>
-      </c>
-      <c r="P5" t="str">
-        <v>Taxa Atual</v>
-      </c>
-      <c r="S5" t="str">
-        <v>NTNB 2029</v>
-      </c>
-      <c r="T5">
-        <v>0.079702</v>
-      </c>
-    </row>
-    <row r="6">
+      <c r="BN5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="BO5" s="2">
+        <v>0.0755</v>
+      </c>
+      <c r="BQ5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="BR5" s="2">
+        <v>0.074766</v>
+      </c>
+      <c r="BS5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="BT5">
+        <v>0.075099</v>
+      </c>
+      <c r="BU5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="BV5">
+        <v>0.075076</v>
+      </c>
+      <c r="BW5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="BX5">
+        <v>0.07503</v>
+      </c>
+      <c r="BY5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="BZ5">
+        <v>0.074062</v>
+      </c>
+      <c r="CA5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="CB5">
+        <v>0.073823</v>
+      </c>
+      <c r="CC5" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="CD5">
+        <v>0.07434400000000001</v>
+      </c>
+    </row>
+    <row r="6" ht="18.75" customHeight="1">
       <c r="C6" t="str">
         <v>NTNB 2028</v>
       </c>
@@ -1010,11 +1445,137 @@
       <c r="S6" t="str">
         <v>NTNB 2030</v>
       </c>
-      <c r="T6">
-        <v>0.0812</v>
-      </c>
-    </row>
-    <row r="7">
+      <c r="T6" s="2">
+        <v>0.076</v>
+      </c>
+      <c r="W6" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="X6" s="2">
+        <v>0.0822</v>
+      </c>
+      <c r="AA6" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="AB6" s="2">
+        <v>0.0778</v>
+      </c>
+      <c r="AE6" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="AF6" s="2">
+        <v>0.0778</v>
+      </c>
+      <c r="AH6" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="AI6" s="2">
+        <v>0.076</v>
+      </c>
+      <c r="AL6" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="AM6" s="2">
+        <v>0.0789</v>
+      </c>
+      <c r="AP6" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="AQ6" s="2">
+        <v>0.0805</v>
+      </c>
+      <c r="AS6" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="AT6" s="2">
+        <v>0.0816</v>
+      </c>
+      <c r="AV6" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="AW6" s="2">
+        <v>0.0862</v>
+      </c>
+      <c r="AY6" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="AZ6" s="2">
+        <v>0.0863</v>
+      </c>
+      <c r="BB6" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="BC6" s="2">
+        <v>0.0833</v>
+      </c>
+      <c r="BE6" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="BF6" s="2">
+        <v>0.0828</v>
+      </c>
+      <c r="BH6" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="BI6" s="2">
+        <v>0.0818</v>
+      </c>
+      <c r="BK6" t="str">
+        <v>NTNB 2029</v>
+      </c>
+      <c r="BL6" s="2">
+        <v>0.079702</v>
+      </c>
+      <c r="BN6" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="BO6" s="2">
+        <v>0.077</v>
+      </c>
+      <c r="BQ6" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="BR6" s="2">
+        <v>0.07655</v>
+      </c>
+      <c r="BS6" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="BT6">
+        <v>0.07586999999999999</v>
+      </c>
+      <c r="BU6" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="BV6">
+        <v>0.0761</v>
+      </c>
+      <c r="BW6" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="BX6">
+        <v>0.0765</v>
+      </c>
+      <c r="BY6" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="BZ6">
+        <v>0.07556</v>
+      </c>
+      <c r="CA6" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="CB6">
+        <v>0.0756</v>
+      </c>
+      <c r="CC6" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="CD6">
+        <v>0.076058</v>
+      </c>
+    </row>
+    <row r="7" ht="18.75" customHeight="1">
       <c r="C7" t="str">
         <v>NTNB 2029</v>
       </c>
@@ -1042,11 +1603,137 @@
       <c r="S7" t="str">
         <v>NTNB 2032</v>
       </c>
-      <c r="T7">
-        <v>0.0809</v>
-      </c>
-    </row>
-    <row r="8">
+      <c r="T7" s="2">
+        <v>0.0748</v>
+      </c>
+      <c r="W7" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="X7" s="2">
+        <v>0.0807</v>
+      </c>
+      <c r="AA7" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="AB7" s="2">
+        <v>0.0773</v>
+      </c>
+      <c r="AE7" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="AF7" s="2">
+        <v>0.0766</v>
+      </c>
+      <c r="AH7" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="AI7" s="2">
+        <v>0.0746</v>
+      </c>
+      <c r="AL7" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="AM7" s="2">
+        <v>0.0775</v>
+      </c>
+      <c r="AP7" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="AQ7" s="2">
+        <v>0.0793</v>
+      </c>
+      <c r="AS7" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="AT7" s="2">
+        <v>0.0803</v>
+      </c>
+      <c r="AV7" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="AW7" s="2">
+        <v>0.0847</v>
+      </c>
+      <c r="AY7" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="AZ7" s="2">
+        <v>0.0834</v>
+      </c>
+      <c r="BB7" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="BC7" s="2">
+        <v>0.0817</v>
+      </c>
+      <c r="BE7" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="BF7" s="2">
+        <v>0.0821</v>
+      </c>
+      <c r="BH7" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="BI7" s="2">
+        <v>0.0817</v>
+      </c>
+      <c r="BK7" t="str">
+        <v>NTNB 2030</v>
+      </c>
+      <c r="BL7" s="2">
+        <v>0.0812</v>
+      </c>
+      <c r="BN7" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="BO7" s="2">
+        <v>0.0775</v>
+      </c>
+      <c r="BQ7" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="BR7" s="2">
+        <v>0.076431</v>
+      </c>
+      <c r="BS7" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="BT7">
+        <v>0.075816</v>
+      </c>
+      <c r="BU7" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="BV7">
+        <v>0.076483</v>
+      </c>
+      <c r="BW7" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="BX7">
+        <v>0.07685</v>
+      </c>
+      <c r="BY7" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="BZ7">
+        <v>0.076072</v>
+      </c>
+      <c r="CA7" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="CB7">
+        <v>0.076347</v>
+      </c>
+      <c r="CC7" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="CD7">
+        <v>0.076197</v>
+      </c>
+    </row>
+    <row r="8" ht="18.75" customHeight="1">
       <c r="C8" t="str">
         <v>NTNB 2030</v>
       </c>
@@ -1074,11 +1761,137 @@
       <c r="S8" t="str">
         <v>NTNB 2035</v>
       </c>
-      <c r="T8">
-        <v>0.079372</v>
-      </c>
-    </row>
-    <row r="9">
+      <c r="T8" s="2">
+        <v>0.0735</v>
+      </c>
+      <c r="W8" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="X8" s="2">
+        <v>0.0781</v>
+      </c>
+      <c r="AA8" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="AB8" s="2">
+        <v>0.076</v>
+      </c>
+      <c r="AE8" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="AF8" s="2">
+        <v>0.0752</v>
+      </c>
+      <c r="AH8" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="AI8" s="2">
+        <v>0.0729</v>
+      </c>
+      <c r="AL8" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="AM8" s="2">
+        <v>0.0758</v>
+      </c>
+      <c r="AP8" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="AQ8" s="2">
+        <v>0.0772</v>
+      </c>
+      <c r="AS8" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="AT8" s="2">
+        <v>0.0785</v>
+      </c>
+      <c r="AV8" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="AW8" s="2">
+        <v>0.0813</v>
+      </c>
+      <c r="AY8" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="AZ8" s="2">
+        <v>0.0816</v>
+      </c>
+      <c r="BB8" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="BC8" s="2">
+        <v>0.0805</v>
+      </c>
+      <c r="BE8" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="BF8" s="2">
+        <v>0.0809</v>
+      </c>
+      <c r="BH8" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="BI8" s="2">
+        <v>0.0802</v>
+      </c>
+      <c r="BK8" t="str">
+        <v>NTNB 2032</v>
+      </c>
+      <c r="BL8" s="2">
+        <v>0.0809</v>
+      </c>
+      <c r="BN8" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="BO8" s="2">
+        <v>0.0772</v>
+      </c>
+      <c r="BQ8" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="BR8" s="2">
+        <v>0.076099</v>
+      </c>
+      <c r="BS8" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="BT8">
+        <v>0.075543</v>
+      </c>
+      <c r="BU8" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="BV8">
+        <v>0.076182</v>
+      </c>
+      <c r="BW8" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="BX8">
+        <v>0.07635900000000001</v>
+      </c>
+      <c r="BY8" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="BZ8">
+        <v>0.076111</v>
+      </c>
+      <c r="CA8" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="CB8">
+        <v>0.0764</v>
+      </c>
+      <c r="CC8" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="CD8">
+        <v>0.076169</v>
+      </c>
+    </row>
+    <row r="9" ht="19.5" customHeight="1">
       <c r="C9" t="str">
         <v>NTNB 2032</v>
       </c>
@@ -1106,8 +1919,134 @@
       <c r="S9" t="str">
         <v>NTNB 2045</v>
       </c>
-      <c r="T9">
-        <v>0.075538</v>
+      <c r="T9" s="2">
+        <v>0.0706</v>
+      </c>
+      <c r="W9" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="X9" s="2">
+        <v>0.0747</v>
+      </c>
+      <c r="AA9" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="AB9" s="2">
+        <v>0.0728</v>
+      </c>
+      <c r="AE9" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="AF9" s="2">
+        <v>0.072</v>
+      </c>
+      <c r="AH9" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="AI9" s="2">
+        <v>0.0704</v>
+      </c>
+      <c r="AL9" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="AM9" s="2">
+        <v>0.0724</v>
+      </c>
+      <c r="AP9" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="AQ9" s="2">
+        <v>0.0737</v>
+      </c>
+      <c r="AS9" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="AT9" s="2">
+        <v>0.0747</v>
+      </c>
+      <c r="AV9" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="AW9" s="2">
+        <v>0.0761</v>
+      </c>
+      <c r="AY9" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="AZ9" s="2">
+        <v>0.0775</v>
+      </c>
+      <c r="BB9" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="BC9" s="2">
+        <v>0.0758</v>
+      </c>
+      <c r="BE9" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="BF9" s="2">
+        <v>0.0765</v>
+      </c>
+      <c r="BH9" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="BI9" s="2">
+        <v>0.0761</v>
+      </c>
+      <c r="BK9" t="str">
+        <v>NTNB 2035</v>
+      </c>
+      <c r="BL9" s="2">
+        <v>0.079372</v>
+      </c>
+      <c r="BN9" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="BO9" s="2">
+        <v>0.0747</v>
+      </c>
+      <c r="BQ9" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="BR9" s="2">
+        <v>0.0736</v>
+      </c>
+      <c r="BS9" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="BT9">
+        <v>0.073659</v>
+      </c>
+      <c r="BU9" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="BV9">
+        <v>0.0739</v>
+      </c>
+      <c r="BW9" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="BX9">
+        <v>0.074067</v>
+      </c>
+      <c r="BY9" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="BZ9">
+        <v>0.07381599999999999</v>
+      </c>
+      <c r="CA9" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="CB9">
+        <v>0.07400000000000001</v>
+      </c>
+      <c r="CC9" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="CD9">
+        <v>0.0738</v>
       </c>
     </row>
     <row r="10">
@@ -1134,6 +2073,12 @@
       </c>
       <c r="P10" s="2">
         <v>0.075</v>
+      </c>
+      <c r="BK10" t="str">
+        <v>NTNB 2045</v>
+      </c>
+      <c r="BL10" s="2">
+        <v>0.075538</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -1165,7 +2110,7 @@
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="C2:T11"/>
+    <ignoredError numberStoredAsText="1" sqref="C2:CD11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>